<commit_message>
Fix empty sheet dependency
</commit_message>
<xml_diff>
--- a/demo.xlsx
+++ b/demo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/elga3498_colorado_edu/Documents/Documents/cu/crdds/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="13_ncr:1_{86884339-B6B9-4345-A3D8-F3EE94B4CEE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1ADAFD28-FB1F-2A42-B381-EFD5AE3865C3}"/>
+  <xr:revisionPtr revIDLastSave="124" documentId="13_ncr:1_{86884339-B6B9-4345-A3D8-F3EE94B4CEE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48250610-842F-F34B-83D6-F93686717BCD}"/>
   <bookViews>
-    <workbookView xWindow="76780" yWindow="1680" windowWidth="25600" windowHeight="28180" activeTab="9" xr2:uid="{CB725B27-3C12-D848-9427-6C443DCCCD5D}"/>
+    <workbookView xWindow="51740" yWindow="1660" windowWidth="25600" windowHeight="28180" activeTab="8" xr2:uid="{CB725B27-3C12-D848-9427-6C443DCCCD5D}"/>
   </bookViews>
   <sheets>
     <sheet name="upper_left_corner" sheetId="3" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="63">
   <si>
     <t>a</t>
   </si>
@@ -231,6 +231,9 @@
   </si>
   <si>
     <t>6</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -305,10 +308,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -691,7 +690,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1525FC60-3619-1A4B-B469-23E77BFA782A}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -757,6 +756,11 @@
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D6" t="s">
+        <v>62</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1832,4 +1836,10 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{3ded8b1b-070d-4629-82e4-c0b019f46057}" enabled="0" method="" siteId="{3ded8b1b-070d-4629-82e4-c0b019f46057}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Adding tests and updating documentation
Added two tests: delimiter matches extension and check for whitespace in headers. Added headers with whitespace to demo.xlsx. Updated Test_Suite to open tsv in addition to csv using pandas read_csv. Also updated README with new tests and some other minor changes.
</commit_message>
<xml_diff>
--- a/demo.xlsx
+++ b/demo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/elga3498_colorado_edu/Documents/Documents/cu/crdds/excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ap180/Automated-Spreadsheet-Curation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="124" documentId="13_ncr:1_{86884339-B6B9-4345-A3D8-F3EE94B4CEE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48250610-842F-F34B-83D6-F93686717BCD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20141F98-4119-EE4D-98D3-B186510AA59B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51740" yWindow="1660" windowWidth="25600" windowHeight="28180" activeTab="8" xr2:uid="{CB725B27-3C12-D848-9427-6C443DCCCD5D}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17640" activeTab="3" xr2:uid="{CB725B27-3C12-D848-9427-6C443DCCCD5D}"/>
   </bookViews>
   <sheets>
     <sheet name="upper_left_corner" sheetId="3" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="65">
   <si>
     <t>a</t>
   </si>
@@ -234,6 +234,12 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> header-leading</t>
+  </si>
+  <si>
+    <t xml:space="preserve">header-trailing </t>
   </si>
 </sst>
 </file>
@@ -1387,10 +1393,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC1D4482-C0E4-544B-91B2-4C02764184A1}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1415,8 +1421,14 @@
       <c r="I1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J1" t="s">
+        <v>64</v>
+      </c>
+      <c r="K1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1444,8 +1456,14 @@
       <c r="I2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1473,8 +1491,14 @@
       <c r="I3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1502,8 +1526,14 @@
       <c r="I4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1531,8 +1561,14 @@
       <c r="I5">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1560,8 +1596,14 @@
       <c r="I6">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J6">
+        <v>5</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>66</v>
       </c>
@@ -1587,6 +1629,12 @@
         <v>66</v>
       </c>
       <c r="I7">
+        <v>66</v>
+      </c>
+      <c r="J7">
+        <v>66</v>
+      </c>
+      <c r="K7">
         <v>66</v>
       </c>
     </row>

</xml_diff>